<commit_message>
Extractor done, new format for json file
</commit_message>
<xml_diff>
--- a/refactor/menu_template.xlsx
+++ b/refactor/menu_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25427"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My MacBook Pro\Documents\programmation\python\menu\menu v2.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mastalp\Documents\menu\refactor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{142149D7-E760-4D2B-BEBB-4A3987589CF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21FE85FB-D698-4552-A7EC-CBD41DA1FC9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6465" yWindow="5535" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="menu_template" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="16">
   <si>
     <t>FR</t>
   </si>
@@ -202,7 +202,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -430,11 +430,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -523,10 +543,6 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -575,6 +591,10 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="14" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -605,7 +625,19 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -1772,7 +1804,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:IV13"/>
+  <dimension ref="A1:IV15"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="18" style="1" customWidth="1"/>
@@ -1783,7 +1815,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:256" s="3" customFormat="1" ht="50.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="38" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="5"/>
@@ -2255,11 +2287,11 @@
       <c r="A8" s="18"/>
       <c r="B8" s="19"/>
       <c r="C8" s="20"/>
-      <c r="D8" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>6</v>
+      <c r="D8" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" s="50" t="s">
+        <v>5</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="17"/>
@@ -2277,40 +2309,40 @@
       <c r="S8" s="17"/>
     </row>
     <row r="9" spans="1:256" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="E9" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="F9" s="25"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="16"/>
       <c r="G9" s="17"/>
-      <c r="H9" s="25"/>
+      <c r="H9" s="16"/>
       <c r="I9" s="17"/>
-      <c r="J9" s="25"/>
+      <c r="J9" s="16"/>
       <c r="K9" s="17"/>
-      <c r="L9" s="25"/>
-      <c r="M9" s="26"/>
-      <c r="N9" s="25"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="17"/>
+      <c r="N9" s="16"/>
       <c r="O9" s="17"/>
-      <c r="P9" s="25"/>
+      <c r="P9" s="16"/>
       <c r="Q9" s="17"/>
-      <c r="R9" s="25"/>
+      <c r="R9" s="16"/>
       <c r="S9" s="17"/>
     </row>
-    <row r="10" spans="1:256" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="27"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="29"/>
+    <row r="10" spans="1:256" ht="65.099999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>14</v>
+      </c>
       <c r="D10" s="23" t="s">
         <v>2</v>
       </c>
@@ -2329,18 +2361,18 @@
       <c r="O10" s="17"/>
       <c r="P10" s="25"/>
       <c r="Q10" s="17"/>
-      <c r="R10" s="25"/>
+      <c r="R10" s="36"/>
       <c r="S10" s="17"/>
     </row>
-    <row r="11" spans="1:256" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="30"/>
-      <c r="B11" s="31"/>
-      <c r="C11" s="29"/>
+    <row r="11" spans="1:256" ht="65.099999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="26"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="28"/>
       <c r="D11" s="23" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E11" s="24" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F11" s="25"/>
       <c r="G11" s="17"/>
@@ -2349,18 +2381,18 @@
       <c r="J11" s="25"/>
       <c r="K11" s="17"/>
       <c r="L11" s="25"/>
-      <c r="M11" s="26"/>
+      <c r="M11" s="17"/>
       <c r="N11" s="25"/>
       <c r="O11" s="17"/>
       <c r="P11" s="25"/>
       <c r="Q11" s="17"/>
-      <c r="R11" s="25"/>
+      <c r="R11" s="36"/>
       <c r="S11" s="17"/>
     </row>
-    <row r="12" spans="1:256" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="30"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="29"/>
+    <row r="12" spans="1:256" ht="65.099999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="29"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="28"/>
       <c r="D12" s="23" t="s">
         <v>4</v>
       </c>
@@ -2374,38 +2406,88 @@
       <c r="J12" s="25"/>
       <c r="K12" s="17"/>
       <c r="L12" s="25"/>
-      <c r="M12" s="26"/>
+      <c r="M12" s="17"/>
       <c r="N12" s="25"/>
       <c r="O12" s="17"/>
       <c r="P12" s="25"/>
       <c r="Q12" s="17"/>
-      <c r="R12" s="25"/>
+      <c r="R12" s="36"/>
       <c r="S12" s="17"/>
     </row>
     <row r="13" spans="1:256" ht="65.099999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
-      <c r="B13" s="33"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="35" t="s">
+      <c r="A13" s="29"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="F13" s="25"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="25"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="25"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="25"/>
+      <c r="M13" s="17"/>
+      <c r="N13" s="25"/>
+      <c r="O13" s="17"/>
+      <c r="P13" s="25"/>
+      <c r="Q13" s="17"/>
+      <c r="R13" s="36"/>
+      <c r="S13" s="17"/>
+    </row>
+    <row r="14" spans="1:256" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="29"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="51" t="s">
+        <v>4</v>
+      </c>
+      <c r="E14" s="52" t="s">
+        <v>5</v>
+      </c>
+      <c r="F14" s="25"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="25"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="25"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="25"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="25"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="36"/>
+      <c r="S14" s="17"/>
+    </row>
+    <row r="15" spans="1:256" ht="53.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="31"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="E13" s="36" t="s">
+      <c r="E15" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="F13" s="37"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="38"/>
-      <c r="J13" s="37"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="37"/>
-      <c r="M13" s="17"/>
-      <c r="N13" s="37"/>
-      <c r="O13" s="17"/>
-      <c r="P13" s="37"/>
-      <c r="Q13" s="17"/>
-      <c r="R13" s="37"/>
-      <c r="S13" s="17"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="37"/>
+      <c r="J15" s="36"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="36"/>
+      <c r="M15" s="17"/>
+      <c r="N15" s="36"/>
+      <c r="O15" s="17"/>
+      <c r="P15" s="36"/>
+      <c r="Q15" s="17"/>
+      <c r="R15" s="36"/>
+      <c r="S15" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>